<commit_message>
docs: alinear alcance web y retirar foro de planificación
Actualiza informe, visión y backlog, requisitos, historias, Gantt y arquitectura. Incorpora HU18/RF-28 educativa como planificada con detalle y estimación pendientes; distingue avisos internos y decisiones pendientes. Actualiza índices de documentación.
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/Pethub_Requisitos_Funcionales_y_No_Funcionales.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/Pethub_Requisitos_Funcionales_y_No_Funcionales.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requisitos Pethub" sheetId="1" r:id="Raecbb8b9e1b04025"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requisitos Pethub" sheetId="1" r:id="Rb9eccf2cb9ab49a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -42,7 +42,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
         <x:fgColor rgb="FF946138"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF1F1F1"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -86,7 +91,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="19">
+  <x:cellXfs count="21">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -139,6 +144,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -398,9 +409,9 @@
         <x:v>PETHUB | Requisitos funcionales y no funcionales</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="24" customHeight="1">
+    <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Fuente: Pethub_Historias_Usuario_3.xlsx · 17 historias de usuario y sus 51 escenarios de aceptación. E = escenario.</x:v>
+        <x:v>Alcance web ajustado según reunión del 15-10-2026. HU15–HU17 y RF23–RF27: retirados. HU18 / RF28: sección educativa, detalle por validar.</x:v>
       </x:c>
       <x:c r="B2" s="3" t="str">
         <x:v>Fuente: Pethub_Historias_Usuario_3.xlsx · 17 historias de usuario y sus 51 escenarios de aceptación. E = escenario.</x:v>
@@ -418,9 +429,9 @@
         <x:v>Fuente: Pethub_Historias_Usuario_3.xlsx · 17 historias de usuario y sus 51 escenarios de aceptación. E = escenario.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="27" customHeight="1">
+    <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>Alcance: especificación del sistema esperado; no certifica funciones implementadas. Los requisitos o métricas propuestos requieren validación del equipo.</x:v>
+        <x:v>Estado: carnet sanitario y red de donantes se mantienen; avisos dentro de la web. Chat, correo y nuevos módulos de la práctica: por definir. No certifica implementación.</x:v>
       </x:c>
       <x:c r="B3" s="3" t="str">
         <x:v>Alcance: especificación del sistema esperado; no certifica funciones implementadas. Los requisitos o métricas propuestos requieren validación del equipo.</x:v>
@@ -646,44 +657,44 @@
         <x:v>Derivado de HU</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="92" customHeight="1">
+    <x:row r="15" ht="72" customHeight="1">
       <x:c r="A15" s="15" t="str">
         <x:v>RF-08</x:v>
       </x:c>
       <x:c r="B15" s="13" t="str">
-        <x:v>Recordatorios de vacunas</x:v>
+        <x:v>Recordatorios de vacunas en la web</x:v>
       </x:c>
       <x:c r="C15" s="13" t="str">
-        <x:v>Revisar diariamente los refuerzos y enviar un recordatorio push con tres días de anticipación.</x:v>
+        <x:v>Consultar dentro de la plataforma los recordatorios de refuerzos próximos. El envío push deja de ser requisito de esta entrega.</x:v>
       </x:c>
       <x:c r="D15" s="13" t="str">
         <x:v>S2-HU07 · E1 y E3</x:v>
       </x:c>
       <x:c r="E15" s="13" t="str">
-        <x:v>Se notifica un refuerzo previsto dentro de 3 días; una vacuna marcada como aplicada no genera recordatorio.</x:v>
+        <x:v>Un refuerzo próximo genera un recordatorio visible en la web; las vacunas aplicadas se excluyen.</x:v>
       </x:c>
       <x:c r="F15" s="13" t="str">
-        <x:v>Derivado de HU</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="92" customHeight="1">
+        <x:v>Ajuste de alcance · HU07</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="72" customHeight="1">
       <x:c r="A16" s="14" t="str">
         <x:v>RF-09</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>Recordatorio alternativo en la app</x:v>
+        <x:v>Consulta de recordatorios pendientes</x:v>
       </x:c>
       <x:c r="C16" s="12" t="str">
-        <x:v>Registrar el intento fallido de push cuando no hay permisos y mostrar el recordatorio al iniciar sesión.</x:v>
+        <x:v>Mostrar los recordatorios pendientes en Inicio, sin requerir permisos push del dispositivo.</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
         <x:v>S2-HU07 · E2</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
-        <x:v>Con push desactivado, el usuario encuentra el recordatorio pendiente dentro de la aplicación.</x:v>
+        <x:v>El usuario encuentra los recordatorios al consultar Inicio. Correo: por definir.</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
-        <x:v>Derivado de HU</x:v>
+        <x:v>Ajuste de alcance · HU07</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="92" customHeight="1">
@@ -800,30 +811,30 @@
         <x:v>S4-HU11 · E2</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
-        <x:v>Un donante no disponible no recibe el push de una nueva solicitud coincidente.</x:v>
+        <x:v>Por definir: la regla de disponibilidad y su edición no se declaran terminadas. No se exige envío push.</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
-        <x:v>Derivado de HU</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="92" customHeight="1">
+        <x:v>Por definir · no comprometido</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="85" customHeight="1">
       <x:c r="A23" s="15" t="str">
         <x:v>RF-16</x:v>
       </x:c>
       <x:c r="B23" s="13" t="str">
-        <x:v>Alertas de solicitudes</x:v>
+        <x:v>Avisos de solicitudes dentro de la web</x:v>
       </x:c>
       <x:c r="C23" s="13" t="str">
-        <x:v>Enviar push mediante Firebase Cloud Messaging a todos los dueños de donantes disponibles cuya especie y grupo coincidan con la solicitud.</x:v>
+        <x:v>Crear avisos internos para dueños de donantes coincidentes por especie y grupo; permitir consultarlos, filtrar no leídos y marcarlos como leídos.</x:v>
       </x:c>
       <x:c r="D23" s="13" t="str">
         <x:v>S4-HU11 · E1–E3</x:v>
       </x:c>
       <x:c r="E23" s="13" t="str">
-        <x:v>La publicación dispara avisos a todos los destinatarios elegibles, sin priorizar a uno sobre otro.</x:v>
+        <x:v>La solicitud coincidente genera el aviso; el marcado se conserva al recargar. No exige FCM, permisos push ni entrega con el navegador cerrado.</x:v>
       </x:c>
       <x:c r="F23" s="13" t="str">
-        <x:v>Derivado de HU</x:v>
+        <x:v>Ajuste web · HU11</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="92" customHeight="1">
@@ -831,7 +842,7 @@
         <x:v>RF-17</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
-        <x:v>Contacto directo</x:v>
+        <x:v>POR DEFINIR · Contacto directo</x:v>
       </x:c>
       <x:c r="C24" s="12" t="str">
         <x:v>Abrir un chat interno entre el solicitante y el dueño del donante mediante Contactar.</x:v>
@@ -843,7 +854,7 @@
         <x:v>El contacto válido abre la conversación; una solicitud resuelta impide iniciar un nuevo chat e informa su estado.</x:v>
       </x:c>
       <x:c r="F24" s="12" t="str">
-        <x:v>Derivado de HU</x:v>
+        <x:v>Dependiente del alcance de contacto/chat</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="92" customHeight="1">
@@ -851,7 +862,7 @@
         <x:v>RF-18</x:v>
       </x:c>
       <x:c r="B25" s="13" t="str">
-        <x:v>Restricción por bloqueo de usuario</x:v>
+        <x:v>POR DEFINIR · Restricción por bloqueo de usuario</x:v>
       </x:c>
       <x:c r="C25" s="13" t="str">
         <x:v>Impedir iniciar un chat cuando una de las partes haya bloqueado a la otra.</x:v>
@@ -863,7 +874,7 @@
         <x:v>El intento de contacto no abre el chat y muestra que no es posible contactar al usuario.</x:v>
       </x:c>
       <x:c r="F25" s="13" t="str">
-        <x:v>Derivado de HU</x:v>
+        <x:v>Dependiente del alcance de contacto/chat</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="92" customHeight="1">
@@ -891,7 +902,7 @@
         <x:v>RF-20</x:v>
       </x:c>
       <x:c r="B27" s="13" t="str">
-        <x:v>Mensajería en tiempo real</x:v>
+        <x:v>POR DEFINIR · Mensajería en tiempo real</x:v>
       </x:c>
       <x:c r="C27" s="13" t="str">
         <x:v>Enviar y recibir mensajes dentro de la conversación entre ambos usuarios.</x:v>
@@ -903,7 +914,7 @@
         <x:v>Un mensaje enviado se muestra en ambas conversaciones sin necesidad de recargar manualmente.</x:v>
       </x:c>
       <x:c r="F27" s="13" t="str">
-        <x:v>Derivado de HU</x:v>
+        <x:v>Dependiente del alcance de contacto/chat</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="92" customHeight="1">
@@ -911,7 +922,7 @@
         <x:v>RF-21</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
-        <x:v>Reintento de mensajes sin conexión</x:v>
+        <x:v>POR DEFINIR · Reintento de mensajes sin conexión</x:v>
       </x:c>
       <x:c r="C28" s="12" t="str">
         <x:v>Mantener el mensaje pendiente, informar la falta de conexión y reintentar el envío al recuperarla.</x:v>
@@ -923,7 +934,7 @@
         <x:v>Al desconectar y reconectar, el mensaje pendiente se envía automáticamente.</x:v>
       </x:c>
       <x:c r="F28" s="12" t="str">
-        <x:v>Derivado de HU</x:v>
+        <x:v>Dependiente del alcance de contacto/chat</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="92" customHeight="1">
@@ -931,7 +942,7 @@
         <x:v>RF-22</x:v>
       </x:c>
       <x:c r="B29" s="13" t="str">
-        <x:v>Historial del chat</x:v>
+        <x:v>POR DEFINIR · Historial del chat</x:v>
       </x:c>
       <x:c r="C29" s="13" t="str">
         <x:v>Recuperar el historial completo de la conversación después de cerrar y volver a abrir la aplicación.</x:v>
@@ -943,116 +954,128 @@
         <x:v>Los mensajes anteriores siguen disponibles y conservan su orden de envío.</x:v>
       </x:c>
       <x:c r="F29" s="13" t="str">
-        <x:v>Derivado de HU</x:v>
+        <x:v>Dependiente del alcance de contacto/chat</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="92" customHeight="1">
-      <x:c r="A30" s="14" t="str">
+      <x:c r="A30" s="19" t="str">
         <x:v>RF-23</x:v>
       </x:c>
-      <x:c r="B30" s="12" t="str">
-        <x:v>Publicación en el foro</x:v>
-      </x:c>
-      <x:c r="C30" s="12" t="str">
-        <x:v>Permitir publicar preguntas o experiencias con título y contenido; listar las publicaciones por fecha.</x:v>
-      </x:c>
-      <x:c r="D30" s="12" t="str">
+      <x:c r="B30" s="20" t="str">
+        <x:v>RETIRADO · Publicación en el foro</x:v>
+      </x:c>
+      <x:c r="C30" s="20" t="str">
+        <x:v>Fuera del alcance vigente: Permitir publicar preguntas o experiencias con título y contenido; listar las publicaciones por fecha.</x:v>
+      </x:c>
+      <x:c r="D30" s="20" t="str">
         <x:v>S5-HU15 · E1–E2</x:v>
       </x:c>
-      <x:c r="E30" s="12" t="str">
-        <x:v>Una publicación válida aparece en el listado; sin contenido se muestra un error y no se crea.</x:v>
-      </x:c>
-      <x:c r="F30" s="12" t="str">
-        <x:v>Derivado de HU</x:v>
+      <x:c r="E30" s="20" t="str">
+        <x:v>No exigible en la entrega web. Se conserva la referencia histórica; reemplazado por sección educativa (RF-28).</x:v>
+      </x:c>
+      <x:c r="F30" s="20" t="str">
+        <x:v>Retirado · acuerdo 15-10-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="92" customHeight="1">
-      <x:c r="A31" s="15" t="str">
+      <x:c r="A31" s="19" t="str">
         <x:v>RF-24</x:v>
       </x:c>
-      <x:c r="B31" s="13" t="str">
-        <x:v>Eliminación de publicación propia</x:v>
-      </x:c>
-      <x:c r="C31" s="13" t="str">
-        <x:v>Eliminar una publicación propia y sus comentarios asociados, previa confirmación.</x:v>
-      </x:c>
-      <x:c r="D31" s="13" t="str">
+      <x:c r="B31" s="20" t="str">
+        <x:v>RETIRADO · Eliminación de publicación propia</x:v>
+      </x:c>
+      <x:c r="C31" s="20" t="str">
+        <x:v>Fuera del alcance vigente: Eliminar una publicación propia y sus comentarios asociados, previa confirmación.</x:v>
+      </x:c>
+      <x:c r="D31" s="20" t="str">
         <x:v>S5-HU15 · E3</x:v>
       </x:c>
-      <x:c r="E31" s="13" t="str">
-        <x:v>Al confirmar se eliminan la publicación y sus comentarios; al cancelar se conservan.</x:v>
-      </x:c>
-      <x:c r="F31" s="13" t="str">
-        <x:v>Derivado de HU</x:v>
+      <x:c r="E31" s="20" t="str">
+        <x:v>No exigible en la entrega web. Se conserva la referencia histórica; reemplazado por sección educativa (RF-28).</x:v>
+      </x:c>
+      <x:c r="F31" s="20" t="str">
+        <x:v>Retirado · acuerdo 15-10-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="92" customHeight="1">
-      <x:c r="A32" s="14" t="str">
+      <x:c r="A32" s="19" t="str">
         <x:v>RF-25</x:v>
       </x:c>
-      <x:c r="B32" s="12" t="str">
-        <x:v>Comentarios en el foro</x:v>
-      </x:c>
-      <x:c r="C32" s="12" t="str">
-        <x:v>Permitir comentar publicaciones existentes y mostrar los comentarios a los usuarios del foro.</x:v>
-      </x:c>
-      <x:c r="D32" s="12" t="str">
+      <x:c r="B32" s="20" t="str">
+        <x:v>RETIRADO · Comentarios en el foro</x:v>
+      </x:c>
+      <x:c r="C32" s="20" t="str">
+        <x:v>Fuera del alcance vigente: Permitir comentar publicaciones existentes y mostrar los comentarios a los usuarios del foro.</x:v>
+      </x:c>
+      <x:c r="D32" s="20" t="str">
         <x:v>S5-HU16 · E1–E2</x:v>
       </x:c>
-      <x:c r="E32" s="12" t="str">
-        <x:v>El comentario con texto aparece debajo de la publicación; un comentario vacío se rechaza.</x:v>
-      </x:c>
-      <x:c r="F32" s="12" t="str">
-        <x:v>Derivado de HU</x:v>
+      <x:c r="E32" s="20" t="str">
+        <x:v>No exigible en la entrega web. Se conserva la referencia histórica; reemplazado por sección educativa (RF-28).</x:v>
+      </x:c>
+      <x:c r="F32" s="20" t="str">
+        <x:v>Retirado · acuerdo 15-10-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="92" customHeight="1">
-      <x:c r="A33" s="15" t="str">
+      <x:c r="A33" s="19" t="str">
         <x:v>RF-26</x:v>
       </x:c>
-      <x:c r="B33" s="13" t="str">
-        <x:v>Reporte de comentarios</x:v>
-      </x:c>
-      <x:c r="C33" s="13" t="str">
-        <x:v>Registrar reportes, confirmar su recepción y ocultar automáticamente comentarios con tres o más reportes.</x:v>
-      </x:c>
-      <x:c r="D33" s="13" t="str">
+      <x:c r="B33" s="20" t="str">
+        <x:v>RETIRADO · Reporte de comentarios</x:v>
+      </x:c>
+      <x:c r="C33" s="20" t="str">
+        <x:v>Fuera del alcance vigente: Registrar reportes, confirmar su recepción y ocultar automáticamente comentarios con tres o más reportes.</x:v>
+      </x:c>
+      <x:c r="D33" s="20" t="str">
         <x:v>S5-HU16 · E3</x:v>
       </x:c>
-      <x:c r="E33" s="13" t="str">
-        <x:v>El comentario queda oculto al alcanzar 3 reportes. La HU no define cómo tratar reportes repetidos del mismo usuario.</x:v>
-      </x:c>
-      <x:c r="F33" s="13" t="str">
-        <x:v>Derivado de HU</x:v>
+      <x:c r="E33" s="20" t="str">
+        <x:v>No exigible en la entrega web. Se conserva la referencia histórica; reemplazado por sección educativa (RF-28).</x:v>
+      </x:c>
+      <x:c r="F33" s="20" t="str">
+        <x:v>Retirado · acuerdo 15-10-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="92" customHeight="1">
-      <x:c r="A34" s="14" t="str">
+      <x:c r="A34" s="19" t="str">
         <x:v>RF-27</x:v>
       </x:c>
-      <x:c r="B34" s="12" t="str">
-        <x:v>Búsqueda en el foro</x:v>
-      </x:c>
-      <x:c r="C34" s="12" t="str">
-        <x:v>Buscar palabras en título o contenido, con un mínimo de tres caracteres, y ordenar coincidencias por fecha.</x:v>
-      </x:c>
-      <x:c r="D34" s="12" t="str">
+      <x:c r="B34" s="20" t="str">
+        <x:v>RETIRADO · Búsqueda en el foro</x:v>
+      </x:c>
+      <x:c r="C34" s="20" t="str">
+        <x:v>Fuera del alcance vigente: Buscar palabras en título o contenido, con un mínimo de tres caracteres, y ordenar coincidencias por fecha.</x:v>
+      </x:c>
+      <x:c r="D34" s="20" t="str">
         <x:v>S5-HU17 · E1–E3</x:v>
       </x:c>
-      <x:c r="E34" s="12" t="str">
-        <x:v>Se muestran coincidencias; sin resultados se sugieren alternativas; con menos de 3 caracteres no se busca.</x:v>
-      </x:c>
-      <x:c r="F34" s="12" t="str">
-        <x:v>Derivado de HU</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="3"/>
-      <x:c r="B35" s="3"/>
-      <x:c r="C35" s="3"/>
-      <x:c r="D35" s="3"/>
-      <x:c r="E35" s="3"/>
-      <x:c r="F35" s="3"/>
+      <x:c r="E34" s="20" t="str">
+        <x:v>No exigible en la entrega web. Se conserva la referencia histórica; reemplazado por sección educativa (RF-28).</x:v>
+      </x:c>
+      <x:c r="F34" s="20" t="str">
+        <x:v>Retirado · acuerdo 15-10-2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="85" customHeight="1">
+      <x:c r="A35" s="3" t="str">
+        <x:v>RF-28</x:v>
+      </x:c>
+      <x:c r="B35" s="3" t="str">
+        <x:v>Sección educativa</x:v>
+      </x:c>
+      <x:c r="C35" s="3" t="str">
+        <x:v>Incorporar una sección web de contenido educativo para tutores, en reemplazo del foro.</x:v>
+      </x:c>
+      <x:c r="D35" s="3" t="str">
+        <x:v>S5-HU18</x:v>
+      </x:c>
+      <x:c r="E35" s="3" t="str">
+        <x:v>Contenido, responsable de validación y criterios detallados pendientes de acuerdo. No incluye publicaciones ni comentarios de usuarios.</x:v>
+      </x:c>
+      <x:c r="F35" s="3" t="str">
+        <x:v>Reemplazo acordado · detalle por validar</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="30" customHeight="1">
       <x:c r="A36" s="18" t="str">
@@ -1125,7 +1148,7 @@
         <x:v>Proteger registros sanitarios y conversaciones frente al acceso de otros usuarios no autorizados.</x:v>
       </x:c>
       <x:c r="D39" s="13" t="str">
-        <x:v>S1-HU02; S1-HU03; S2-HU06; S5-HU14</x:v>
+        <x:v>S1-HU02; S1-HU03; S2-HU06; chat excluido hasta definir alcance</x:v>
       </x:c>
       <x:c r="E39" s="13" t="str">
         <x:v>Con dos cuentas, intentar leer o modificar datos privados de la otra por interfaz y API; todos los intentos deben denegarse.</x:v>
@@ -1145,7 +1168,7 @@
         <x:v>Almacenar contraseñas con hash y sal; proteger el intercambio de datos mediante conexiones cifradas.</x:v>
       </x:c>
       <x:c r="D40" s="12" t="str">
-        <x:v>S1-HU01; S1-HU02; S5-HU14</x:v>
+        <x:v>S1-HU01; S1-HU02; chat excluido hasta definir alcance</x:v>
       </x:c>
       <x:c r="E40" s="12" t="str">
         <x:v>Revisar almacenamiento y tráfico: no debe haber contraseñas en texto plano ni transmisión de datos privados sin cifrado.</x:v>
@@ -1179,7 +1202,7 @@
         <x:v>RNF-05</x:v>
       </x:c>
       <x:c r="B42" s="12" t="str">
-        <x:v>Persistencia de conversaciones</x:v>
+        <x:v>POR DEFINIR · Persistencia de conversaciones</x:v>
       </x:c>
       <x:c r="C42" s="12" t="str">
         <x:v>Conservar completo y ordenado el historial tras cerrar y reabrir la aplicación.</x:v>
@@ -1191,7 +1214,7 @@
         <x:v>Enviar varios mensajes, cerrar y reabrir: todos deben recuperarse en el mismo orden.</x:v>
       </x:c>
       <x:c r="F42" s="12" t="str">
-        <x:v>Explícito en HU</x:v>
+        <x:v>Dependiente del alcance de contacto/chat</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="92" customHeight="1">
@@ -1199,7 +1222,7 @@
         <x:v>RNF-06</x:v>
       </x:c>
       <x:c r="B43" s="13" t="str">
-        <x:v>Tolerancia a interrupciones</x:v>
+        <x:v>POR DEFINIR · Tolerancia a interrupciones</x:v>
       </x:c>
       <x:c r="C43" s="13" t="str">
         <x:v>Recuperar el envío de mensajes ante pérdida de conexión sin pérdida ni duplicación de mensajes.</x:v>
@@ -1211,7 +1234,7 @@
         <x:v>Interrumpir la red durante el envío y restaurarla; el mensaje debe entregarse una sola vez. La ausencia de duplicados es una precisión propuesta.</x:v>
       </x:c>
       <x:c r="F43" s="13" t="str">
-        <x:v>Derivado · por validar</x:v>
+        <x:v>Dependiente del alcance de contacto/chat</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="92" customHeight="1">
@@ -1219,7 +1242,7 @@
         <x:v>RNF-07</x:v>
       </x:c>
       <x:c r="B44" s="12" t="str">
-        <x:v>Rendimiento del chat</x:v>
+        <x:v>POR DEFINIR · Rendimiento del chat</x:v>
       </x:c>
       <x:c r="C44" s="12" t="str">
         <x:v>Entregar mensajes en tiempo real con un umbral medible para la prueba del proyecto.</x:v>
@@ -1231,7 +1254,7 @@
         <x:v>Meta propuesta: al menos 95 de 100 mensajes entregados en ≤2 segundos con 20 usuarios conectados y red estable; validar capacidad y entorno.</x:v>
       </x:c>
       <x:c r="F44" s="12" t="str">
-        <x:v>Propuesto · por validar</x:v>
+        <x:v>Dependiente del alcance de contacto/chat</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="92" customHeight="1">
@@ -1242,13 +1265,13 @@
         <x:v>Rendimiento de búsquedas</x:v>
       </x:c>
       <x:c r="C45" s="13" t="str">
-        <x:v>Responder a las búsquedas de donantes y publicaciones dentro de un tiempo aceptable para el usuario.</x:v>
+        <x:v>Responder a las búsquedas de donantes dentro de un tiempo aceptable. La búsqueda del foro se retira.</x:v>
       </x:c>
       <x:c r="D45" s="13" t="str">
-        <x:v>S3-HU10; S5-HU17</x:v>
+        <x:v>S3-HU10</x:v>
       </x:c>
       <x:c r="E45" s="13" t="str">
-        <x:v>Meta propuesta: 95 de 100 búsquedas en ≤3 segundos con 1.000 registros por módulo, 20 usuarios concurrentes y red estable.</x:v>
+        <x:v>Meta propuesta: 95 de 100 búsquedas en ≤3 segundos con 1.000 registros y 20 usuarios concurrentes; entorno y umbral por validar.</x:v>
       </x:c>
       <x:c r="F45" s="13" t="str">
         <x:v>Propuesto · por validar</x:v>
@@ -1265,7 +1288,7 @@
         <x:v>Presentar mensajes en español que expliquen el problema y la corrección requerida, sin perder innecesariamente lo ingresado.</x:v>
       </x:c>
       <x:c r="D46" s="12" t="str">
-        <x:v>S1-HU01; S2-HU04; S2-HU06; S3-HU10; S5-HU17</x:v>
+        <x:v>HU del alcance web vigente</x:v>
       </x:c>
       <x:c r="E46" s="12" t="str">
         <x:v>Revisar casos inválidos: cada uno muestra una explicación y acción de corrección. Conservar campos válidos es una mejora propuesta.</x:v>
@@ -1279,16 +1302,16 @@
         <x:v>RNF-10</x:v>
       </x:c>
       <x:c r="B47" s="13" t="str">
-        <x:v>Compatibilidad de la interfaz móvil</x:v>
+        <x:v>Compatibilidad web adaptable</x:v>
       </x:c>
       <x:c r="C47" s="13" t="str">
-        <x:v>Permitir completar los flujos de mascotas, donación y chat en pantallas móviles sin controles cortados.</x:v>
+        <x:v>Permitir usar los flujos del alcance web en navegador de escritorio y móvil, sin controles cortados.</x:v>
       </x:c>
       <x:c r="D47" s="13" t="str">
-        <x:v>S1-HU03; S3-HU08–HU10; S4-HU12; S5-HU14</x:v>
+        <x:v>HU del alcance web vigente</x:v>
       </x:c>
       <x:c r="E47" s="13" t="str">
-        <x:v>Meta propuesta: verificar flujos en anchos de 360 y 390 px, sin desplazamiento horizontal. Acordar dispositivos y versiones de sistemas soportados.</x:v>
+        <x:v>Propuesta: verificar anchos de 360, 390 y 1280 px, sin desplazamiento horizontal; navegadores soportados por validar.</x:v>
       </x:c>
       <x:c r="F47" s="13" t="str">
         <x:v>Propuesto · por validar</x:v>
@@ -1305,7 +1328,7 @@
         <x:v>Contar con respaldo recuperable de cuentas, carnets, solicitudes y conversaciones.</x:v>
       </x:c>
       <x:c r="D48" s="12" t="str">
-        <x:v>S1-HU01; S2-HU04–HU06; S3-HU09; S5-HU14</x:v>
+        <x:v>S1-HU01; S2-HU04–HU06; S3-HU09; chat excluido hasta definir alcance</x:v>
       </x:c>
       <x:c r="E48" s="12" t="str">
         <x:v>Meta propuesta: respaldo diario y restauración de prueba con pérdida máxima de 24 horas; validar frecuencia y tiempo de recuperación.</x:v>
@@ -1333,8 +1356,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab3e9e3129ba424c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a5bbdf1007c4124"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f9b8a9d7b2c426b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cae62c9f18346d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>